<commit_message>
Mise à jour site panneaux rocko
</commit_message>
<xml_diff>
--- a/prix/prix.xlsx
+++ b/prix/prix.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\caisse5\Desktop\pages-GitHub Braconnier\panneaux-rocko\prix\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\panneaux-rocko\prix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EA98D2F-9497-45BD-9591-5E98D7E9B13F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50EA36B4-4E83-4A40-A610-D2224A3C4C55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="276" yWindow="1068" windowWidth="19116" windowHeight="10884" xr2:uid="{6E95DC93-531D-460D-9A06-44397A8920D7}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="19416" windowHeight="11016" xr2:uid="{6E95DC93-531D-460D-9A06-44397A8920D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -311,10 +311,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -696,13 +696,13 @@
       <c r="C2" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="27">
-        <v>206.04</v>
+      <c r="D2" s="26">
+        <v>237.26</v>
       </c>
       <c r="E2" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="26">
+      <c r="F2" s="27">
         <v>4</v>
       </c>
     </row>
@@ -716,13 +716,13 @@
       <c r="C3" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="27">
-        <v>206.04</v>
+      <c r="D3" s="26">
+        <v>237.26</v>
       </c>
       <c r="E3" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="26">
+      <c r="F3" s="27">
         <v>4</v>
       </c>
     </row>
@@ -736,14 +736,14 @@
       <c r="C4" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="27">
-        <v>206.04</v>
+      <c r="D4" s="26">
+        <v>237.26</v>
       </c>
       <c r="E4" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="26">
-        <v>10</v>
+      <c r="F4" s="27">
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -756,13 +756,13 @@
       <c r="C5" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="27">
-        <v>206.04</v>
+      <c r="D5" s="26">
+        <v>237.26</v>
       </c>
       <c r="E5" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="26">
+      <c r="F5" s="27">
         <v>5</v>
       </c>
     </row>
@@ -776,13 +776,13 @@
       <c r="C6" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="27">
-        <v>206.04</v>
+      <c r="D6" s="26">
+        <v>237.26</v>
       </c>
       <c r="E6" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="26">
+      <c r="F6" s="27">
         <v>6.2100000000000009</v>
       </c>
     </row>
@@ -796,13 +796,13 @@
       <c r="C7" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D7" s="27">
-        <v>206.04</v>
+      <c r="D7" s="26">
+        <v>237.26</v>
       </c>
       <c r="E7" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="26">
+      <c r="F7" s="27">
         <v>6</v>
       </c>
     </row>
@@ -816,14 +816,14 @@
       <c r="C8" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="27">
-        <v>206.04</v>
+      <c r="D8" s="26">
+        <v>237.26</v>
       </c>
       <c r="E8" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="F8" s="26">
-        <v>5</v>
+      <c r="F8" s="27">
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -836,13 +836,13 @@
       <c r="C9" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="27">
-        <v>206.04</v>
+      <c r="D9" s="26">
+        <v>237.26</v>
       </c>
       <c r="E9" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="26">
+      <c r="F9" s="27">
         <v>4</v>
       </c>
     </row>
@@ -856,13 +856,13 @@
       <c r="C10" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="27">
-        <v>206.04</v>
+      <c r="D10" s="26">
+        <v>237.26</v>
       </c>
       <c r="E10" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="F10" s="26">
+      <c r="F10" s="27">
         <v>5</v>
       </c>
     </row>
@@ -876,13 +876,13 @@
       <c r="C11" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="27">
-        <v>206.04</v>
+      <c r="D11" s="26">
+        <v>237.26</v>
       </c>
       <c r="E11" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="F11" s="26">
+      <c r="F11" s="27">
         <v>3</v>
       </c>
     </row>

</xml_diff>